<commit_message>
20250703 - minor typos and updates SoE
Minor typos were corrected.
SoE tables were updated with assessments based on the new studies (e.g., mechanistic) and reordering of figures in the cells.
</commit_message>
<xml_diff>
--- a/data_u1/soe_tables_2025.01.16.xlsx
+++ b/data_u1/soe_tables_2025.01.16.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sksiafis/Desktop/LSR3_taar1_H_2025.04.01/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sksiafis/Documents/GitHub/LSR3_taar1_H/data_u1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{620122FE-400E-2949-9593-B69E13AEB10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF96FD0C-09D8-EC43-B82D-EC4956CAB120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22380" yWindow="-21100" windowWidth="27640" windowHeight="20020" firstSheet="1" activeTab="9" xr2:uid="{5B3852FF-2BEC-B94D-907F-9BD79E8D9C2A}"/>
+    <workbookView xWindow="16680" yWindow="-20700" windowWidth="37260" windowHeight="20020" xr2:uid="{5B3852FF-2BEC-B94D-907F-9BD79E8D9C2A}"/>
   </bookViews>
   <sheets>
     <sheet name="sch_ac_ta1_pl_eff" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="262">
   <si>
     <t>Outcome</t>
   </si>
@@ -74,21 +74,9 @@
     <t>Depressive symptoms (PANSS anxiety/depression factor) (Figure 6)</t>
   </si>
   <si>
-    <t>Overall symptoms (PANSS total) – primary outcome (Figure 40)</t>
-  </si>
-  <si>
     <t>N=1, n=214; 7.9% vs. 13.5%, OR=0.55, 95%CI: 0.22, 1.35</t>
   </si>
   <si>
-    <t>Positive symptoms (PANSS positive subscale/factor) (Figure 41)</t>
-  </si>
-  <si>
-    <t>Negative symptoms (PANSS negative subscale/factor) (Figure 42)</t>
-  </si>
-  <si>
-    <t>Depressive symptoms (PANSS anxiety/depression factor) (Figure 43)</t>
-  </si>
-  <si>
     <t>6 weeks</t>
   </si>
   <si>
@@ -155,21 +143,12 @@
     <t>N=1 n=69; 15.3% vs. 1.4%, OR=12.44, 95%CI: 0.66, 234.38</t>
   </si>
   <si>
-    <t>Hypotension (Figure 20)</t>
-  </si>
-  <si>
     <t>N=1 n=39; 52.4% vs. 78.6%, OR=0.3, 95%CI: 0.07, 1.32</t>
   </si>
   <si>
-    <t>Dizziness (Figure 21)</t>
-  </si>
-  <si>
     <t>Dizziness (Figure 22)</t>
   </si>
   <si>
-    <t>Nausea/vomitting (Figure 23)</t>
-  </si>
-  <si>
     <t>Nausea/vomitting (Figure 24)</t>
   </si>
   <si>
@@ -179,36 +158,21 @@
     <t>N=1 n=245; not estimable effect size 0 events in both arms</t>
   </si>
   <si>
-    <t>QTc interval (msec) (Figure 26)</t>
-  </si>
-  <si>
     <t>N=1 n=62; MD=1.25, 95%CI: -2.87, 5.37</t>
   </si>
   <si>
-    <t>Weight (kg) (Figure 28)</t>
-  </si>
-  <si>
     <t>N=1 n=245; MD=0.4, 95%CI: -0.13, 0.93</t>
   </si>
   <si>
     <t>N=1 n=24; not estimable effect size 0 events in both arms</t>
   </si>
   <si>
-    <t>Prolactin levels (ng/ml) (Figure 29)</t>
-  </si>
-  <si>
     <t>N=1 n=227; MD=-0.58, 95%CI: -7.87, 6.7</t>
   </si>
   <si>
-    <t>Akathisia (Figure 30)</t>
-  </si>
-  <si>
     <t>N=1 n=245; 1.2% vs. 0.4%, OR=3.15, 95%CI: 0.13, 78.11</t>
   </si>
   <si>
-    <t>Extrapyramidal symptoms (Figure 31)</t>
-  </si>
-  <si>
     <t>N=1 n=245; 3.3% vs. 3.2%, OR=1.04, 95%CI: 0.25, 4.27</t>
   </si>
   <si>
@@ -218,39 +182,15 @@
     <t>N=1 n=69; not estimable effect size 0 events in both arms</t>
   </si>
   <si>
-    <t>Anxiety (Figure 32)</t>
-  </si>
-  <si>
-    <t>Agitation (Figure 33)</t>
-  </si>
-  <si>
-    <t>Headache (Figure 33)</t>
-  </si>
-  <si>
     <t>N=1 n=69; 11.5% vs. 20.6%, OR=0.5, 95%CI: 0.13, 1.89</t>
   </si>
   <si>
-    <t>Headache (Figure 34)</t>
-  </si>
-  <si>
-    <t>Sedation (Figure 36)</t>
-  </si>
-  <si>
     <t>Sedation (Figure 37)</t>
   </si>
   <si>
-    <t>Insomnia (Figure 38)</t>
-  </si>
-  <si>
-    <t>Dropouts due to any reason (Figure 46)</t>
-  </si>
-  <si>
     <t>N=1 n=71; 14.3% vs. 5.6%, OR=2.83, 95%CI: 0.51, 15.69</t>
   </si>
   <si>
-    <t>Dropouts due to any reason (Figure 47)</t>
-  </si>
-  <si>
     <t>N=1 n=214; 22.9% vs. 18.9%, OR=1.27, 95%CI: 0.63, 2.56</t>
   </si>
   <si>
@@ -260,57 +200,30 @@
     <t>N=1 n=71; not estimable effect size 0 events in both arms</t>
   </si>
   <si>
-    <t>Dropouts due to adverse events (Figure 48)</t>
-  </si>
-  <si>
     <t>N=1 n=214; 6.4% vs. 1.4%, OR=5.02, 95%CI: 0.62, 40.38</t>
   </si>
   <si>
-    <t>Serious adverse events (Figure 49)</t>
-  </si>
-  <si>
-    <t>Serious adverse events (Figure 50)</t>
-  </si>
-  <si>
     <t>N=1 n=214; 2.5% vs. 0.7%, OR=3.79, 95%CI: 0.19, 74.42</t>
   </si>
   <si>
     <t>N=1 n=214; not estimable effect size 0 events in both arms</t>
   </si>
   <si>
-    <t>Any adverse event (Figure 51)</t>
-  </si>
-  <si>
-    <t>Any adverse event (Figure 52)</t>
-  </si>
-  <si>
     <t>N=1 n=214; 26.5% vs. 48.6%, OR=0.38, 95%CI: 0.21, 0.68</t>
   </si>
   <si>
-    <t>Anticholinergic symptom (Figure 53)</t>
-  </si>
-  <si>
     <t>N=1 n=71; 15.3% vs. 1.4%, OR=13.16, 95%CI: 0.7, 247.71</t>
   </si>
   <si>
-    <t>Dizziness (Figure 54)</t>
-  </si>
-  <si>
     <t>N=1 n=214; 1.4% vs. 8.1%, OR=0.16, 95%CI: 0.03, 0.84</t>
   </si>
   <si>
     <t>N=1 n=214; 1.4% vs. 10.8%, OR=0.12, 95%CI: 0.02, 0.58</t>
   </si>
   <si>
-    <t>Anxiety (Figure 58)</t>
-  </si>
-  <si>
     <t>N=1 n=71; 1.2% vs. 8.3%, OR=0.13, 95%CI: 0.01, 2.71</t>
   </si>
   <si>
-    <t>Anxiety (Figure 59)</t>
-  </si>
-  <si>
     <t>N=1 n=214; 3.6% vs. 6.8%, OR=0.51, 95%CI: 0.14, 1.83</t>
   </si>
   <si>
@@ -338,21 +251,6 @@
     <t>N=1, n=156; SMD=-0.23, 95%CI: -0.56, 0.1</t>
   </si>
   <si>
-    <t>Agitation (Figure 60)</t>
-  </si>
-  <si>
-    <t>Headache (Figure 61)</t>
-  </si>
-  <si>
-    <t>Headache (Figure 62)</t>
-  </si>
-  <si>
-    <t>Sedation (Figure 63)</t>
-  </si>
-  <si>
-    <t>Insomnia (Figure 64)</t>
-  </si>
-  <si>
     <t>Other biases</t>
   </si>
   <si>
@@ -398,15 +296,9 @@
     <t>Low risk: 1 study with an overall low risk of bias.</t>
   </si>
   <si>
-    <t>Overall symptoms (NPI) (Figure 1b)</t>
-  </si>
-  <si>
     <t>Response to treatment (≥50% in SAPS-PD) (Figure 8b)</t>
   </si>
   <si>
-    <t>Positive symptoms (SAPS-PD) (Figure 2b)</t>
-  </si>
-  <si>
     <t>Low risk: 75% had overall low risk of bias.</t>
   </si>
   <si>
@@ -461,27 +353,12 @@
     <t>N=2, n=399; Random-effects: SMD=0.17, 95%CI: -0.06, 0.39; Fixed-effects: SMD=0.17, 95%CI: -0.03, 0.37</t>
   </si>
   <si>
-    <t>Nausea/vomiting (Figure 55)</t>
-  </si>
-  <si>
-    <t>Nausea/vomiting (Figure 56)</t>
-  </si>
-  <si>
-    <t>QTc prolongation (any cut-off) (Figure 25)</t>
-  </si>
-  <si>
     <t>QTc prolongation (any cut-off)</t>
   </si>
   <si>
-    <t>Weight increased (≥7% increase or any cut-off) (Figure 27)</t>
-  </si>
-  <si>
     <t>Prolactin elevation (any cut-off)</t>
   </si>
   <si>
-    <t>Weight increased (any cut-off) (Figure 57)</t>
-  </si>
-  <si>
     <t>Death due to any cause</t>
   </si>
   <si>
@@ -491,12 +368,6 @@
     <t>N=1, n=96; In anticipation of loss, ulotaront appeared to be associated with smaller BOLD striatal responses compared to placebo (left: SMD=-0.55, 95%CI: -1.05, -0.05; right: SMD=-0.44, 95%CI: -0.94, 0.06) but not to amisulpride (left: SMD=-0.22, 95%CI: -0.71, 0.27; right: SMD: -0.11, 95%CI: -0.60, 0.38). In anticipation of a win, ulotaront did not seem to differ in BOLD striatal responses compared to placebo (left: SMD=-0.25, 95%CI: -0.75, 0.25; right: SMD=-0.25, 95%CI: -0.75, 0.25) and amisulpride (left: SMD=-0.11, 95%CI: -0.60, 0.38; right: SMD=-0.08, 95%CI: -0.57, 0.41). The interaction with schizotypy traits for BOLD striatal responses was not reported. However, it was reported that ulotaront could reverse, in comparison to placebo, the aberrant BOLD right insular responses to anticipation of loss in participants with high schizotypy traits.</t>
   </si>
   <si>
-    <t>N=4, n=1291; Random-effects: SMD=0.15, 95%CI: -0.05, 0.34; Fixed-effects: SMD=0.13, 95%CI: 0.02, 0.25; Dose effects: uncertain/unclear dose-response indication (Figure 67)</t>
-  </si>
-  <si>
-    <t>Response to treatment (≥50%reduction in PANSS total) (Figure 44)</t>
-  </si>
-  <si>
     <t>Moderate risk: Three trials were conducted during COVID-19 (2 in ulotaront, 1 in ralmitaront), which in some cases could be associated with factors related to smaller effect sizes. Specifically, a pooled analysis of the two Phase III ulotaront trials, using only the participants enrolled before COVID-19, showed effect sizes like the Phase II ulotaront trial. This may have underestimated the effects of TAAR1 agonists compared to placebo in favor of the latter.</t>
   </si>
   <si>
@@ -542,13 +413,7 @@
     <t>Moderate risk: Ulotaront appeared to cause sedation in 60% of the participants, more frequently compared to placebo (Figure 36) and amisulpride (Figure 63). Consequently, ulotaront was associated with decreased performance and accuracy across the different neuropsychological tasks used in the study, but it was not correlated with the BOLD responses and impaired reaction times by &lt;10% in this task. The impact of this bias on the magnitude and direction of the effects of TAAR1 agonists on this outcome is unclear.</t>
   </si>
   <si>
-    <t>Negative symptoms (BNSS or PANSS negative subscale/factor) (Figure 5)</t>
-  </si>
-  <si>
     <t>N=2 n=399; Random-effects: SMD=0.27, 95%CI: -0.06, 0.59; Fixed-effecs: SMD=0.29, 95%CI: 0.09, 0.49</t>
-  </si>
-  <si>
-    <t>Relapse (schizophrenia as adverse eventl) (Figure 44)</t>
   </si>
   <si>
     <t>52 weeks</t>
@@ -571,15 +436,9 @@
     </r>
   </si>
   <si>
-    <t>Relapse (dropout due to relapse) (Figure 8a)</t>
-  </si>
-  <si>
     <t>12 weeks</t>
   </si>
   <si>
-    <t>N=1 n=16; SMD=0.44, 95%CI: -0.58, 1.47; Dose effects: uncertain/unclear dose-response indication (Figure 67)</t>
-  </si>
-  <si>
     <t>N=1 n=27; 2.7% vs. 6.7%, OR=0.39, 95%CI: 0.01, 10.37</t>
   </si>
   <si>
@@ -592,18 +451,6 @@
     <t>Negative symptoms (PANSS negative factor) (Figure 5)</t>
   </si>
   <si>
-    <t>Positive symptoms (PANSS positive factor) (Figure 4a)</t>
-  </si>
-  <si>
-    <t>N=1 n=16; SMD=0.13, 95%CI: -0.88, 1.15; Dose effects: uncertain/unclear dose-response indication (Figure 67)</t>
-  </si>
-  <si>
-    <t>Response to treatment (≥50% reduction in PANSS total) (Figure 8a)</t>
-  </si>
-  <si>
-    <t>N=1 n=76; SMD=0.26, 95%CI: -0.2, 0.72; Dose effects: uncertain/unclear dose-response indication (Figure 67)</t>
-  </si>
-  <si>
     <t>N=1 n=104; 10.4% vs. 10.8%, OR=0.96, 95%CI: 0.26, 3.53</t>
   </si>
   <si>
@@ -613,9 +460,6 @@
     <t>N=1 n=76; SMD=0.18, 95%CI: -0.28, 0.64</t>
   </si>
   <si>
-    <t>N=1 n=75; SMD=0.25, 95%CI: -0.22, 0.71; Dose effects: uncertain/unclear dose-response indication (Figure 67)</t>
-  </si>
-  <si>
     <t>4-12 weeks</t>
   </si>
   <si>
@@ -749,13 +593,284 @@
   </si>
   <si>
     <t>N=1 n=104; 1.5% vs. 8.1%, OR=0.17, 95%CI: 0.02, 1.71</t>
+  </si>
+  <si>
+    <t>Overall symptoms (NPI) (Figure 3b)</t>
+  </si>
+  <si>
+    <t>Overall symptoms (PANSS total)  - primary outcome (Figure 3c)</t>
+  </si>
+  <si>
+    <r>
+      <t>High risk: 1 study with overall high risk of bias (due to missing outcome data).</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>The impact of the bias on the magnitude and direction of the effects of TAAR1 agonists is unclear.</t>
+    </r>
+  </si>
+  <si>
+    <t>Positive symptoms (PANSS positive factor) (Figure 4c)</t>
+  </si>
+  <si>
+    <t>Negative symptoms (BNSS or PANSS negative subscale/factor) (Figure 5a)</t>
+  </si>
+  <si>
+    <t>Positive symptoms (SAPS-PD) (Figure 4b)</t>
+  </si>
+  <si>
+    <t>Response to treatment (≥50% reduction in PANSS total) (Figure 8c)</t>
+  </si>
+  <si>
+    <t>Relapse (dropout due to relapse) (Figure 9)</t>
+  </si>
+  <si>
+    <t>Anticholinergic symptom (Figure 20)</t>
+  </si>
+  <si>
+    <t>Hypotension (Figure 21)</t>
+  </si>
+  <si>
+    <t>Dizziness (Figure 23)</t>
+  </si>
+  <si>
+    <t>Nausea/vomitting (Figure 25)</t>
+  </si>
+  <si>
+    <t>QTc prolongation (any cut-off) (Figure 26)</t>
+  </si>
+  <si>
+    <t>QTc interval (msec) (Figure 27)</t>
+  </si>
+  <si>
+    <t>Weight increased (≥7% increase or any cut-off) (Figure 28)</t>
+  </si>
+  <si>
+    <t>Weight (kg) (Figure 29)</t>
+  </si>
+  <si>
+    <t>Prolactin levels (ng/ml) (Figure 30)</t>
+  </si>
+  <si>
+    <t>Akathisia (Figure 31)</t>
+  </si>
+  <si>
+    <t>Extrapyramidal symptoms (Figure 32)</t>
+  </si>
+  <si>
+    <t>Anxiety (Figure 33)</t>
+  </si>
+  <si>
+    <t>Agitation (Figure 34)</t>
+  </si>
+  <si>
+    <t>Headache (Figure 35)</t>
+  </si>
+  <si>
+    <t>Headache (Figure 36)</t>
+  </si>
+  <si>
+    <t>Sedation (Figure 38)</t>
+  </si>
+  <si>
+    <t>Insomnia (Figure 39)</t>
+  </si>
+  <si>
+    <t>Overall symptoms (PANSS total) – primary outcome (Figure 42)</t>
+  </si>
+  <si>
+    <t>Positive symptoms (PANSS positive subscale/factor) (Figure 43)</t>
+  </si>
+  <si>
+    <t>Negative symptoms (PANSS negative subscale/factor) (Figure 44)</t>
+  </si>
+  <si>
+    <t>Depressive symptoms (PANSS anxiety/depression factor) (Figure 45)</t>
+  </si>
+  <si>
+    <t>Response to treatment (≥50%reduction in PANSS total) (Figure 46)</t>
+  </si>
+  <si>
+    <t>Relapse (schizophrenia as adverse eventl) (Figure 47)</t>
+  </si>
+  <si>
+    <t>Dropouts due to any reason (Figure 48)</t>
+  </si>
+  <si>
+    <t>Dropouts due to any reason (Figure 49)</t>
+  </si>
+  <si>
+    <t>Dropouts due to any reason (Figure 50)</t>
+  </si>
+  <si>
+    <t>Dropouts due to adverse events (Figure 51)</t>
+  </si>
+  <si>
+    <t>Dropouts due to adverse events (Figure 52)</t>
+  </si>
+  <si>
+    <t>Serious adverse events (Figure 53)</t>
+  </si>
+  <si>
+    <t>Serious adverse events (Figure 54)</t>
+  </si>
+  <si>
+    <t>Any adverse event (Figure 55)</t>
+  </si>
+  <si>
+    <t>Any adverse event (Figure 56)</t>
+  </si>
+  <si>
+    <t>Anticholinergic symptom (Figure 57)</t>
+  </si>
+  <si>
+    <t>Anticholinergic symptom (Figure 58)</t>
+  </si>
+  <si>
+    <t>Dizziness (Figure 59)</t>
+  </si>
+  <si>
+    <t>Nausea/vomiting (Figure 60)</t>
+  </si>
+  <si>
+    <t>Nausea/vomiting (Figure 61)</t>
+  </si>
+  <si>
+    <t>Weight increased (any cut-off) (Figure 62)</t>
+  </si>
+  <si>
+    <t>Weight increased (any cut-off) (Figure 63)</t>
+  </si>
+  <si>
+    <t>Weight (kg) (Figure 65)</t>
+  </si>
+  <si>
+    <t>Anxiety (Figure 66)</t>
+  </si>
+  <si>
+    <t>Anxiety (Figure 67)</t>
+  </si>
+  <si>
+    <t>Anxiety (Figure 68)</t>
+  </si>
+  <si>
+    <t>Agitation (Figure 69)</t>
+  </si>
+  <si>
+    <t>Headache (Figure 70)</t>
+  </si>
+  <si>
+    <t>Headache (Figure 71)</t>
+  </si>
+  <si>
+    <t>Sedation (Figure 72)</t>
+  </si>
+  <si>
+    <t>Sedation (Figure 73)</t>
+  </si>
+  <si>
+    <t>Insomnia (Figure 74)</t>
+  </si>
+  <si>
+    <t>Insomnia (Figure 75)</t>
+  </si>
+  <si>
+    <t>Overall symptoms (PANSS total)  - primary outcome (Figure 78)</t>
+  </si>
+  <si>
+    <t>Positive symptoms (PANSS positive factor) (Figure 79)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">High risk: 1 study with overall high risk of bias (due to missing outcome data). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>The impact of the bias on the magnitude and direction of the effects of TAAR1 agonists is unclear.</t>
+    </r>
+  </si>
+  <si>
+    <t>Negative symptoms (PANSS negative factor) (Figure 80)</t>
+  </si>
+  <si>
+    <t>Response to treatment (≥50% reduction in PANSS total) (Figure 81)</t>
+  </si>
+  <si>
+    <t>Relapse (dropout due to relapse)</t>
+  </si>
+  <si>
+    <t>Dropouts due to any reason (Figure 82)</t>
+  </si>
+  <si>
+    <t>Dropouts due to adverse events (Figure 83)</t>
+  </si>
+  <si>
+    <t>Serious adverse events (Figure 84)</t>
+  </si>
+  <si>
+    <t>Death (Figure 85)</t>
+  </si>
+  <si>
+    <t>Any adverse event (Figure 86)</t>
+  </si>
+  <si>
+    <t>Anticholinergic symptom (Figure 87)</t>
+  </si>
+  <si>
+    <t>Dizziness (Figure 88)</t>
+  </si>
+  <si>
+    <t>Nausea/vomiting (Figure 89)</t>
+  </si>
+  <si>
+    <t>Headache (Figure 90)</t>
+  </si>
+  <si>
+    <t>Sedation (Figure 91)</t>
+  </si>
+  <si>
+    <t>Insomnia</t>
+  </si>
+  <si>
+    <t>N=4, n=1291; Random-effects: SMD=0.15, 95%CI: -0.05, 0.34; Fixed-effects: SMD=0.13, 95%CI: 0.02, 0.25; Dose effects: uncertain/unclear dose-response indication (Figure 95)</t>
+  </si>
+  <si>
+    <t>N=1 n=16; SMD=0.13, 95%CI: -0.88, 1.15; Dose effects: uncertain/unclear dose-response indication (Figure 96)</t>
+  </si>
+  <si>
+    <t>N=1 n=16; SMD=0.44, 95%CI: -0.58, 1.47; Dose effects: uncertain/unclear dose-response indication (Figure 96)</t>
+  </si>
+  <si>
+    <t>N=1 n=75; SMD=0.25, 95%CI: -0.22, 0.71; Dose effects: uncertain/unclear dose-response indication (Figure 96)</t>
+  </si>
+  <si>
+    <t>N=1 n=76; SMD=0.26, 95%CI: -0.2, 0.72; Dose effects: uncertain/unclear dose-response indication (Figure 96)</t>
+  </si>
+  <si>
+    <t>Moderate risk: The outcome of relapse was defined as "schizophrenia" adverse event. The impact of the bias on the magnitude and direction of the effects of TAAR1 agonists is unclear.</t>
+  </si>
+  <si>
+    <t>High risk. This might have overestimated the changes observed with TAAR1 agonists.</t>
+  </si>
+  <si>
+    <t>High risk. This might have overestimated the effects of TAAR1 agonistsr.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -773,13 +888,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -802,7 +910,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -812,6 +920,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -895,7 +1009,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -909,17 +1023,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -938,11 +1045,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1278,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE69A57-5664-7440-A961-B0C632901626}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="3"/>
@@ -1301,135 +1411,132 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="211" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>111</v>
+      <c r="A2" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>148</v>
+        <v>254</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>150</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="211" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>112</v>
+      <c r="A3" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>150</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="99" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>113</v>
+      <c r="A4" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>136</v>
+        <v>100</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>123</v>
+        <v>87</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="113" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>165</v>
+      <c r="A5" s="6" t="s">
+        <v>183</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>166</v>
+        <v>122</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>124</v>
+        <v>88</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="99" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="175" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>137</v>
+        <v>101</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>124</v>
+        <v>88</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="5"/>
+        <v>81</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1462,62 +1569,62 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="333" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>103</v>
+      <c r="A2" s="6" t="s">
+        <v>69</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>147</v>
+        <v>106</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>261</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>163</v>
+        <v>120</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>164</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="127" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>105</v>
+      <c r="A3" s="6" t="s">
+        <v>71</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>90</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>260</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1529,146 +1636,143 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB0315C3-E44A-0A41-AD94-C01C5B3109CA}">
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="20.5" style="8"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>102</v>
+      <c r="D1" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="126" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F2" s="12" t="s">
+      <c r="A2" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="12" t="s">
-        <v>115</v>
+      <c r="G2" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="126" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F3" s="12" t="s">
+      <c r="A3" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="12" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="126" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F4" s="12" t="s">
+      <c r="G3" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="112" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>115</v>
+      <c r="G4" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="126" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F5" s="12" t="s">
+      <c r="A5" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="12" t="s">
-        <v>115</v>
+      <c r="G5" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="126" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F6" s="12" t="s">
+      <c r="A6" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="12" t="s">
-        <v>115</v>
+      <c r="G6" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1682,141 +1786,141 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="19.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" ht="42" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>102</v>
+      <c r="D1" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="140" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F2" s="12" t="s">
+      <c r="A2" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="12" t="s">
-        <v>115</v>
+      <c r="G2" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="140" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F3" s="12" t="s">
+      <c r="A3" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="12" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="140" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F4" s="12" t="s">
+      <c r="G3" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="126" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>115</v>
+      <c r="G4" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="140" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F5" s="12" t="s">
+      <c r="A5" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="12" t="s">
-        <v>115</v>
+      <c r="G5" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="140" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F6" s="12" t="s">
+      <c r="A6" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="12" t="s">
-        <v>115</v>
+      <c r="G6" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1840,39 +1944,39 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="253" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>167</v>
+      <c r="A2" s="6" t="s">
+        <v>209</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>169</v>
+        <v>124</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>5</v>
+        <v>80</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>259</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1906,131 +2010,131 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>9</v>
+      <c r="A2" s="6" t="s">
+        <v>204</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>149</v>
+      <c r="A3" s="6" t="s">
+        <v>208</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>11</v>
+      <c r="A4" s="6" t="s">
+        <v>205</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>12</v>
+      <c r="A5" s="6" t="s">
+        <v>206</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>13</v>
+      <c r="A6" s="6" t="s">
+        <v>207</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>96</v>
+        <v>67</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2063,108 +2167,108 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="92" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>117</v>
+      <c r="A2" s="6" t="s">
+        <v>179</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>118</v>
+      <c r="A3" s="6" t="s">
+        <v>83</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>119</v>
+      <c r="A4" s="6" t="s">
+        <v>184</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="91" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>18</v>
+      <c r="A5" s="6" t="s">
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2177,7 +2281,7 @@
   <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="15"/>
+    <col min="1" max="1" width="10.83203125" style="12"/>
     <col min="3" max="3" width="22.5" customWidth="1"/>
     <col min="4" max="4" width="26.33203125" customWidth="1"/>
     <col min="5" max="5" width="26.6640625" customWidth="1"/>
@@ -2186,7 +2290,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="29" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2196,798 +2300,798 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="100" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>20</v>
+      <c r="A2" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>159</v>
+        <v>116</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>151</v>
+        <v>108</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>23</v>
+      <c r="A3" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>187</v>
+        <v>135</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>188</v>
+        <v>136</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="99" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>24</v>
+      <c r="A4" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>159</v>
+        <v>116</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>152</v>
+        <v>109</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>27</v>
+      <c r="A5" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>189</v>
+        <v>137</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>28</v>
+      <c r="A6" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>153</v>
+        <v>110</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>30</v>
+      <c r="A7" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>192</v>
+        <v>140</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="90" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>145</v>
+      <c r="A8" s="6" t="s">
+        <v>104</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>153</v>
+        <v>110</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>146</v>
+      <c r="A9" s="6" t="s">
+        <v>105</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>193</v>
+        <v>141</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>32</v>
+      <c r="A10" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>33</v>
-      </c>
       <c r="B11" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>191</v>
+        <v>139</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="104" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>34</v>
+      <c r="A12" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="104" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>34</v>
+      <c r="A13" s="6" t="s">
+        <v>187</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>194</v>
+        <v>142</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="99" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>36</v>
+      <c r="A14" s="6" t="s">
+        <v>188</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>38</v>
+      <c r="A15" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>155</v>
+        <v>93</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>156</v>
+        <v>113</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="87" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>39</v>
+      <c r="A16" s="6" t="s">
+        <v>189</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>195</v>
+        <v>143</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>197</v>
+        <v>145</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="99" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>40</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>34</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>130</v>
+        <v>94</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>152</v>
+        <v>109</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>41</v>
+      <c r="A18" s="6" t="s">
+        <v>190</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>198</v>
+        <v>146</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="139" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>140</v>
+      <c r="A19" s="6" t="s">
+        <v>191</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>157</v>
+        <v>35</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>114</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>141</v>
+      <c r="A20" s="6" t="s">
+        <v>102</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G20" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="127" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" ht="127" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>158</v>
-      </c>
       <c r="E21" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>142</v>
+      <c r="A22" s="6" t="s">
+        <v>193</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>46</v>
+      <c r="A23" s="6" t="s">
+        <v>194</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="84" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>143</v>
+      <c r="A24" s="6" t="s">
+        <v>103</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>49</v>
+      <c r="A25" s="6" t="s">
+        <v>195</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>51</v>
+      <c r="A26" s="6" t="s">
+        <v>196</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
-        <v>53</v>
+      <c r="A27" s="6" t="s">
+        <v>197</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="98" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>55</v>
+      <c r="A28" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
-        <v>57</v>
+      <c r="A29" s="6" t="s">
+        <v>198</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>132</v>
+        <v>96</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>58</v>
+      <c r="A30" s="6" t="s">
+        <v>199</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="85" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>59</v>
+      <c r="A31" s="6" t="s">
+        <v>200</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
-        <v>61</v>
+      <c r="A32" s="6" t="s">
+        <v>201</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>199</v>
+        <v>147</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
-        <v>62</v>
+      <c r="A33" s="6" t="s">
+        <v>46</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C33" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>186</v>
-      </c>
       <c r="C34" s="4" t="s">
-        <v>200</v>
+        <v>148</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
-        <v>64</v>
+      <c r="A35" s="6" t="s">
+        <v>203</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>202</v>
+        <v>150</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>190</v>
+        <v>138</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -3000,7 +3104,7 @@
   <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="14" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="3"/>
     <col min="3" max="3" width="20.83203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="27.83203125" style="3" customWidth="1"/>
@@ -3010,7 +3114,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="29" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3020,283 +3124,283 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>67</v>
+      <c r="A2" s="6" t="s">
+        <v>243</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>223</v>
+        <v>171</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>71</v>
+      <c r="A3" s="6" t="s">
+        <v>244</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>224</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>74</v>
+      <c r="A4" s="6" t="s">
+        <v>245</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>225</v>
+        <v>173</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>145</v>
+      <c r="A5" s="6" t="s">
+        <v>246</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>78</v>
+      <c r="A6" s="6" t="s">
+        <v>247</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>227</v>
+        <v>175</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>80</v>
+      <c r="A7" s="6" t="s">
+        <v>248</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>224</v>
-      </c>
       <c r="D7" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>82</v>
+      <c r="A8" s="6" t="s">
+        <v>249</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>228</v>
+        <v>176</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>139</v>
+      <c r="A9" s="6" t="s">
+        <v>250</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>229</v>
+        <v>177</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>99</v>
+      <c r="A10" s="6" t="s">
+        <v>251</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>230</v>
+        <v>178</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>100</v>
+      <c r="A11" s="6" t="s">
+        <v>252</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>229</v>
+        <v>177</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>101</v>
+      <c r="A12" s="6" t="s">
+        <v>253</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>183</v>
+        <v>132</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D28D98F-934C-324D-A021-B678B5C46157}">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="14" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="3"/>
     <col min="3" max="3" width="20.83203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="27.83203125" style="3" customWidth="1"/>
@@ -3307,7 +3411,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3317,752 +3421,729 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="81" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>65</v>
+      <c r="A2" s="6" t="s">
+        <v>210</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>67</v>
+      <c r="A3" s="6" t="s">
+        <v>211</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>67</v>
+      <c r="A4" s="6" t="s">
+        <v>212</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>203</v>
+        <v>151</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>69</v>
+      <c r="A5" s="6" t="s">
+        <v>49</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>71</v>
+      <c r="A6" s="6" t="s">
+        <v>213</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>71</v>
+      <c r="A7" s="6" t="s">
+        <v>214</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>204</v>
+        <v>152</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="127" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>73</v>
+      <c r="A8" s="6" t="s">
+        <v>215</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>210</v>
+        <v>153</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>158</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>74</v>
+      <c r="A9" s="6" t="s">
+        <v>216</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="127" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>145</v>
+      <c r="A10" s="6" t="s">
+        <v>104</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>210</v>
+        <v>155</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>158</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="85" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>145</v>
+      <c r="A11" s="6" t="s">
+        <v>104</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>77</v>
+      <c r="A12" s="6" t="s">
+        <v>217</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>209</v>
+        <v>156</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>157</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>78</v>
+      <c r="A13" s="6" t="s">
+        <v>218</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>80</v>
+      <c r="A14" s="6" t="s">
+        <v>219</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>80</v>
+      <c r="A15" s="6" t="s">
+        <v>220</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>211</v>
+        <v>159</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>82</v>
+      <c r="A16" s="6" t="s">
+        <v>221</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>209</v>
+        <v>160</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>157</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>138</v>
+      <c r="A17" s="6" t="s">
+        <v>222</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>209</v>
+        <v>161</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>157</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="29" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>139</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>223</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>214</v>
+        <v>56</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>139</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" customFormat="1" ht="139" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>102</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>116</v>
+      <c r="D19" s="5" t="s">
+        <v>169</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F19" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" customFormat="1" ht="139" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>222</v>
-      </c>
       <c r="G20" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>144</v>
+      <c r="A21" s="6" t="s">
+        <v>225</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>84</v>
+        <v>163</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>144</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="29" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>226</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>215</v>
+        <v>162</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="29" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>46</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>227</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>168</v>
+        <v>17</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>214</v>
+        <v>58</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F23" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G23" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="G24" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>87</v>
+      <c r="A25" s="6" t="s">
+        <v>229</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>88</v>
+        <v>164</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>87</v>
+      <c r="A26" s="6" t="s">
+        <v>230</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>216</v>
+        <v>60</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
-        <v>97</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>231</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F27" s="4" t="s">
+      <c r="C28" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G27" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="71" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F28" s="4" t="s">
+      <c r="G28" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="141" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="G28" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="B29" s="4" t="s">
+      <c r="G29" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="C31" s="4" t="s">
-        <v>218</v>
+        <v>61</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
-        <v>101</v>
+      <c r="A32" s="6" t="s">
+        <v>236</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>90</v>
+        <v>167</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="43" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>